<commit_message>
docs: clarify collaborative flow editing and SDK handoff contracts
</commit_message>
<xml_diff>
--- a/AI에이전트/agentic platform/assets/agent-playground-wbs.xlsx
+++ b/AI에이전트/agentic platform/assets/agent-playground-wbs.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" r:id="R5f9ef4f71f2b4c2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="1" r:id="R94f260d76ddd4f58"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -539,7 +539,7 @@
       </x:c>
       <x:c r="E7" s="33" t="str">
         <x:v>Phase0: Stage 검증
-Phase1: 호환 연동</x:v>
+Phase1: 플로우 호환</x:v>
       </x:c>
       <x:c r="F7" s="34" t="str">
         <x:v>연동 보완</x:v>
@@ -563,7 +563,7 @@
 Phase1: 실험 작업본</x:v>
       </x:c>
       <x:c r="F8" s="34" t="str">
-        <x:v>변경 이력·공유</x:v>
+        <x:v>구조 이력·변경 공유</x:v>
       </x:c>
       <x:c r="G8" s="34" t="str">
         <x:v>통합 검증</x:v>
@@ -620,10 +620,10 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="E11" s="34" t="str">
-        <x:v>import·설정 편집</x:v>
+        <x:v>import·플로우 편집</x:v>
       </x:c>
       <x:c r="F11" s="34" t="str">
-        <x:v>시험·결과 화면</x:v>
+        <x:v>플로우 시험·결과 공유</x:v>
       </x:c>
       <x:c r="G11" s="34" t="str">
         <x:v>기획자 시나리오 검증</x:v>
@@ -643,7 +643,7 @@
         <x:v>import·파일 대응</x:v>
       </x:c>
       <x:c r="F12" s="34" t="str">
-        <x:v>변경점·선택 반영</x:v>
+        <x:v>플로우 비교·반영 검토</x:v>
       </x:c>
       <x:c r="G12" s="34" t="str">
         <x:v>개발자 시나리오 검증</x:v>

</xml_diff>